<commit_message>
feat(synoniemen): Excel-breed formaat — slug links, synoniemen horizontaal
- Sync ondersteunt kolom A = PNG/slug en B+ = extra synoniemen; legacy 2-koloms blijft werken
- Seed groepeert JSON per slug met dynamische kolombreedte
- ingredient-synonyms.json opnieuw gesynchroniseerd (zelfde genormaliseerde sleutels)

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/public/images/items/ingredienten_categorieen.xlsx
+++ b/public/images/items/ingredienten_categorieen.xlsx
@@ -2512,1851 +2512,3491 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B230"/>
+  <dimension ref="A1:I120"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Synoniem</v>
+        <v>Afbeelding (png / slug)</v>
       </c>
       <c r="B1" t="str">
-        <v>Slug</v>
+        <v>Synoniem 1</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Synoniem 2</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Synoniem 3</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Synoniem 4</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Synoniem 5</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Synoniem 6</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Synoniem 7</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Synoniem 8</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>aardappelen</v>
+      </c>
+      <c r="B2" t="str">
         <v>aardappel</v>
       </c>
-      <c r="B2" t="str">
-        <v>aardappelen</v>
+      <c r="C2" t="str">
+        <v>aardappels</v>
+      </c>
+      <c r="D2" t="str">
+        <v>aardappeltje</v>
+      </c>
+      <c r="E2" t="str">
+        <v>aardappeltjes</v>
+      </c>
+      <c r="F2" t="str">
+        <v>frietaardappelen</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>aardappels</v>
+        <v>aardbeien</v>
       </c>
       <c r="B3" t="str">
-        <v>aardappelen</v>
+        <v>aardbei</v>
+      </c>
+      <c r="C3" t="str">
+        <v>aardbeien</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>aardappeltje</v>
+        <v>ajuinen</v>
       </c>
       <c r="B4" t="str">
-        <v>aardappelen</v>
+        <v>ajuin</v>
+      </c>
+      <c r="C4" t="str">
+        <v>gesnipperde ui</v>
+      </c>
+      <c r="D4" t="str">
+        <v>ui</v>
+      </c>
+      <c r="E4" t="str">
+        <v>ui gesnipperd</v>
+      </c>
+      <c r="F4" t="str">
+        <v>uien</v>
+      </c>
+      <c r="G4" t="str">
+        <v>uienringen</v>
+      </c>
+      <c r="H4" t="str">
+        <v>uitje</v>
+      </c>
+      <c r="I4" t="str">
+        <v>uitjes</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>aardappeltjes</v>
+        <v>amandelen</v>
       </c>
       <c r="B5" t="str">
-        <v>aardappelen</v>
+        <v>amandel</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>frietaardappelen</v>
+        <v>appels_1</v>
       </c>
       <c r="B6" t="str">
-        <v>aardappelen</v>
+        <v>appel</v>
+      </c>
+      <c r="C6" t="str">
+        <v>appels</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>aardbei</v>
+        <v>arachideolie</v>
       </c>
       <c r="B7" t="str">
-        <v>aardbeien</v>
+        <v>arachide olie</v>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>aardbeien</v>
+        <v>augurken</v>
       </c>
       <c r="B8" t="str">
-        <v>aardbeien</v>
+        <v>augurk</v>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ajuin</v>
+        <v>avocado</v>
       </c>
       <c r="B9" t="str">
-        <v>ajuinen</v>
+        <v>avocado</v>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>gesnipperde ui</v>
+        <v>bananen</v>
       </c>
       <c r="B10" t="str">
-        <v>ajuinen</v>
+        <v>banaan</v>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>ui</v>
+        <v>basilicum</v>
       </c>
       <c r="B11" t="str">
-        <v>ajuinen</v>
+        <v>verse basilicum</v>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ui gesnipperd</v>
+        <v>bieslook</v>
       </c>
       <c r="B12" t="str">
-        <v>ajuinen</v>
+        <v>verse bieslook</v>
+      </c>
+      <c r="C12" t="str">
+        <v/>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
+        <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>uien</v>
+        <v>blik_tomaten</v>
       </c>
       <c r="B13" t="str">
-        <v>ajuinen</v>
+        <v>gepelde tomaten</v>
+      </c>
+      <c r="C13" t="str">
+        <v>ingeblikte tomaten</v>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>uienringen</v>
+        <v>bloemsuiker</v>
       </c>
       <c r="B14" t="str">
-        <v>ajuinen</v>
+        <v>poedersuiker</v>
+      </c>
+      <c r="C14" t="str">
+        <v/>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>uitje</v>
+        <v>bosbessen</v>
       </c>
       <c r="B15" t="str">
-        <v>ajuinen</v>
+        <v>blauwe bes</v>
+      </c>
+      <c r="C15" t="str">
+        <v>blauwe bessen</v>
+      </c>
+      <c r="D15" t="str">
+        <v>bosbes</v>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+      <c r="I15" t="str">
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>uitjes</v>
+        <v>bouillon</v>
       </c>
       <c r="B16" t="str">
-        <v>ajuinen</v>
+        <v>bouillon blokje</v>
+      </c>
+      <c r="C16" t="str">
+        <v/>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+      <c r="I16" t="str">
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>amandel</v>
+        <v>bruine_suiker</v>
       </c>
       <c r="B17" t="str">
-        <v>amandelen</v>
+        <v>basterdsuiker</v>
+      </c>
+      <c r="C17" t="str">
+        <v>bruine suiker</v>
+      </c>
+      <c r="D17" t="str">
+        <v>cassonade</v>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+      <c r="H17" t="str">
+        <v/>
+      </c>
+      <c r="I17" t="str">
+        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>appel</v>
+        <v>butternut</v>
       </c>
       <c r="B18" t="str">
-        <v>appels_1</v>
+        <v>butternut squash</v>
+      </c>
+      <c r="C18" t="str">
+        <v>pompoen</v>
+      </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18" t="str">
+        <v/>
+      </c>
+      <c r="I18" t="str">
+        <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>appels</v>
+        <v>cacao</v>
       </c>
       <c r="B19" t="str">
-        <v>appels_1</v>
+        <v>cacao poeder</v>
+      </c>
+      <c r="C19" t="str">
+        <v>cacaopoeder</v>
+      </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
+      <c r="I19" t="str">
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>arachide olie</v>
+        <v>cappelini</v>
       </c>
       <c r="B20" t="str">
-        <v>arachideolie</v>
+        <v>spaghetti</v>
+      </c>
+      <c r="C20" t="str">
+        <v/>
+      </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
+      <c r="H20" t="str">
+        <v/>
+      </c>
+      <c r="I20" t="str">
+        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>augurk</v>
+        <v>champignons</v>
       </c>
       <c r="B21" t="str">
-        <v>augurken</v>
+        <v>champignon</v>
+      </c>
+      <c r="C21" t="str">
+        <v>paddenstoel</v>
+      </c>
+      <c r="D21" t="str">
+        <v>paddenstoelen</v>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
+      <c r="I21" t="str">
+        <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>avocado</v>
+        <v>chilipepers</v>
       </c>
       <c r="B22" t="str">
-        <v>avocado</v>
+        <v>chili</v>
+      </c>
+      <c r="C22" t="str">
+        <v>chilivlokken</v>
+      </c>
+      <c r="D22" t="str">
+        <v>rode peper</v>
+      </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
+      <c r="G22" t="str">
+        <v/>
+      </c>
+      <c r="H22" t="str">
+        <v/>
+      </c>
+      <c r="I22" t="str">
+        <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>banaan</v>
+        <v>chocolade</v>
       </c>
       <c r="B23" t="str">
-        <v>bananen</v>
+        <v>melkchocolade</v>
+      </c>
+      <c r="C23" t="str">
+        <v>pure chocolade</v>
+      </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
+      <c r="E23" t="str">
+        <v/>
+      </c>
+      <c r="F23" t="str">
+        <v/>
+      </c>
+      <c r="G23" t="str">
+        <v/>
+      </c>
+      <c r="H23" t="str">
+        <v/>
+      </c>
+      <c r="I23" t="str">
+        <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>verse basilicum</v>
+        <v>citroen</v>
       </c>
       <c r="B24" t="str">
-        <v>basilicum</v>
+        <v>citroensap</v>
+      </c>
+      <c r="C24" t="str">
+        <v/>
+      </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
+      <c r="F24" t="str">
+        <v/>
+      </c>
+      <c r="G24" t="str">
+        <v/>
+      </c>
+      <c r="H24" t="str">
+        <v/>
+      </c>
+      <c r="I24" t="str">
+        <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>verse bieslook</v>
+        <v>curry</v>
       </c>
       <c r="B25" t="str">
-        <v>bieslook</v>
+        <v>currypoeder</v>
+      </c>
+      <c r="C25" t="str">
+        <v/>
+      </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
+      <c r="F25" t="str">
+        <v/>
+      </c>
+      <c r="G25" t="str">
+        <v/>
+      </c>
+      <c r="H25" t="str">
+        <v/>
+      </c>
+      <c r="I25" t="str">
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>gepelde tomaten</v>
+        <v>eieren_1</v>
       </c>
       <c r="B26" t="str">
-        <v>blik_tomaten</v>
+        <v>ei</v>
+      </c>
+      <c r="C26" t="str">
+        <v>eieren</v>
+      </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
+      <c r="F26" t="str">
+        <v/>
+      </c>
+      <c r="G26" t="str">
+        <v/>
+      </c>
+      <c r="H26" t="str">
+        <v/>
+      </c>
+      <c r="I26" t="str">
+        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>ingeblikte tomaten</v>
+        <v>frambozen</v>
       </c>
       <c r="B27" t="str">
-        <v>blik_tomaten</v>
+        <v>framboos</v>
+      </c>
+      <c r="C27" t="str">
+        <v/>
+      </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
+      <c r="F27" t="str">
+        <v/>
+      </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
+      <c r="H27" t="str">
+        <v/>
+      </c>
+      <c r="I27" t="str">
+        <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>poedersuiker</v>
+        <v>gedroogde_gist</v>
       </c>
       <c r="B28" t="str">
-        <v>bloemsuiker</v>
+        <v>droge gist</v>
+      </c>
+      <c r="C28" t="str">
+        <v>droogzout</v>
+      </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+      <c r="G28" t="str">
+        <v/>
+      </c>
+      <c r="H28" t="str">
+        <v/>
+      </c>
+      <c r="I28" t="str">
+        <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>blauwe bes</v>
+        <v>gehakt</v>
       </c>
       <c r="B29" t="str">
-        <v>bosbessen</v>
+        <v>gehakt vlees</v>
+      </c>
+      <c r="C29" t="str">
+        <v>rundergehakt</v>
+      </c>
+      <c r="D29" t="str">
+        <v>varkensgehakt</v>
+      </c>
+      <c r="E29" t="str">
+        <v/>
+      </c>
+      <c r="F29" t="str">
+        <v/>
+      </c>
+      <c r="G29" t="str">
+        <v/>
+      </c>
+      <c r="H29" t="str">
+        <v/>
+      </c>
+      <c r="I29" t="str">
+        <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>blauwe bessen</v>
+        <v>gehakte_walnoten</v>
       </c>
       <c r="B30" t="str">
-        <v>bosbessen</v>
+        <v>gehakte noten</v>
+      </c>
+      <c r="C30" t="str">
+        <v/>
+      </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
+      <c r="E30" t="str">
+        <v/>
+      </c>
+      <c r="F30" t="str">
+        <v/>
+      </c>
+      <c r="G30" t="str">
+        <v/>
+      </c>
+      <c r="H30" t="str">
+        <v/>
+      </c>
+      <c r="I30" t="str">
+        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>bosbes</v>
+        <v>gele_paprika</v>
       </c>
       <c r="B31" t="str">
-        <v>bosbessen</v>
+        <v>gele paprika</v>
+      </c>
+      <c r="C31" t="str">
+        <v/>
+      </c>
+      <c r="D31" t="str">
+        <v/>
+      </c>
+      <c r="E31" t="str">
+        <v/>
+      </c>
+      <c r="F31" t="str">
+        <v/>
+      </c>
+      <c r="G31" t="str">
+        <v/>
+      </c>
+      <c r="H31" t="str">
+        <v/>
+      </c>
+      <c r="I31" t="str">
+        <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>bouillon blokje</v>
+        <v>gember</v>
       </c>
       <c r="B32" t="str">
-        <v>bouillon</v>
+        <v>gemberpowder</v>
+      </c>
+      <c r="C32" t="str">
+        <v>verse gember</v>
+      </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
+      <c r="E32" t="str">
+        <v/>
+      </c>
+      <c r="F32" t="str">
+        <v/>
+      </c>
+      <c r="G32" t="str">
+        <v/>
+      </c>
+      <c r="H32" t="str">
+        <v/>
+      </c>
+      <c r="I32" t="str">
+        <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>basterdsuiker</v>
+        <v>geraspte_kaas</v>
       </c>
       <c r="B33" t="str">
-        <v>bruine_suiker</v>
+        <v>geraspte kaas</v>
+      </c>
+      <c r="C33" t="str">
+        <v>gruyere</v>
+      </c>
+      <c r="D33" t="str">
+        <v>gruyère</v>
+      </c>
+      <c r="E33" t="str">
+        <v>kaas</v>
+      </c>
+      <c r="F33" t="str">
+        <v/>
+      </c>
+      <c r="G33" t="str">
+        <v/>
+      </c>
+      <c r="H33" t="str">
+        <v/>
+      </c>
+      <c r="I33" t="str">
+        <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>bruine suiker</v>
+        <v>geraspte_wortelen</v>
       </c>
       <c r="B34" t="str">
-        <v>bruine_suiker</v>
+        <v>geraspte wortel</v>
+      </c>
+      <c r="C34" t="str">
+        <v>geraspte wortels</v>
+      </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
+      <c r="E34" t="str">
+        <v/>
+      </c>
+      <c r="F34" t="str">
+        <v/>
+      </c>
+      <c r="G34" t="str">
+        <v/>
+      </c>
+      <c r="H34" t="str">
+        <v/>
+      </c>
+      <c r="I34" t="str">
+        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>cassonade</v>
+        <v>gerookte_zalm</v>
       </c>
       <c r="B35" t="str">
-        <v>bruine_suiker</v>
+        <v>gerookte zalm</v>
+      </c>
+      <c r="C35" t="str">
+        <v/>
+      </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
+      <c r="F35" t="str">
+        <v/>
+      </c>
+      <c r="G35" t="str">
+        <v/>
+      </c>
+      <c r="H35" t="str">
+        <v/>
+      </c>
+      <c r="I35" t="str">
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>butternut squash</v>
+        <v>ghee</v>
       </c>
       <c r="B36" t="str">
-        <v>butternut</v>
+        <v>geklaarde boter</v>
+      </c>
+      <c r="C36" t="str">
+        <v>ghee</v>
+      </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
+      <c r="F36" t="str">
+        <v/>
+      </c>
+      <c r="G36" t="str">
+        <v/>
+      </c>
+      <c r="H36" t="str">
+        <v/>
+      </c>
+      <c r="I36" t="str">
+        <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>pompoen</v>
+        <v>groene_asperges</v>
       </c>
       <c r="B37" t="str">
-        <v>butternut</v>
+        <v>asperge</v>
+      </c>
+      <c r="C37" t="str">
+        <v>asperges</v>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
+      <c r="F37" t="str">
+        <v/>
+      </c>
+      <c r="G37" t="str">
+        <v/>
+      </c>
+      <c r="H37" t="str">
+        <v/>
+      </c>
+      <c r="I37" t="str">
+        <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>cacao poeder</v>
+        <v>groentenbouillon</v>
       </c>
       <c r="B38" t="str">
-        <v>cacao</v>
+        <v>groentenbouillon</v>
+      </c>
+      <c r="C38" t="str">
+        <v/>
+      </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
+      <c r="E38" t="str">
+        <v/>
+      </c>
+      <c r="F38" t="str">
+        <v/>
+      </c>
+      <c r="G38" t="str">
+        <v/>
+      </c>
+      <c r="H38" t="str">
+        <v/>
+      </c>
+      <c r="I38" t="str">
+        <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>cacaopoeder</v>
+        <v>hagelslag</v>
       </c>
       <c r="B39" t="str">
-        <v>cacao</v>
+        <v>hagelslag</v>
+      </c>
+      <c r="C39" t="str">
+        <v/>
+      </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
+      <c r="E39" t="str">
+        <v/>
+      </c>
+      <c r="F39" t="str">
+        <v/>
+      </c>
+      <c r="G39" t="str">
+        <v/>
+      </c>
+      <c r="H39" t="str">
+        <v/>
+      </c>
+      <c r="I39" t="str">
+        <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>spaghetti</v>
+        <v>hazelnoten</v>
       </c>
       <c r="B40" t="str">
-        <v>cappelini</v>
+        <v>hazelnoot</v>
+      </c>
+      <c r="C40" t="str">
+        <v/>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
+      <c r="F40" t="str">
+        <v/>
+      </c>
+      <c r="G40" t="str">
+        <v/>
+      </c>
+      <c r="H40" t="str">
+        <v/>
+      </c>
+      <c r="I40" t="str">
+        <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>champignon</v>
+        <v>honing</v>
       </c>
       <c r="B41" t="str">
-        <v>champignons</v>
+        <v>honing</v>
+      </c>
+      <c r="C41" t="str">
+        <v>vloeibare honing</v>
+      </c>
+      <c r="D41" t="str">
+        <v/>
+      </c>
+      <c r="E41" t="str">
+        <v/>
+      </c>
+      <c r="F41" t="str">
+        <v/>
+      </c>
+      <c r="G41" t="str">
+        <v/>
+      </c>
+      <c r="H41" t="str">
+        <v/>
+      </c>
+      <c r="I41" t="str">
+        <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>paddenstoel</v>
+        <v>ijsbergsla</v>
       </c>
       <c r="B42" t="str">
-        <v>champignons</v>
+        <v>ijssla</v>
+      </c>
+      <c r="C42" t="str">
+        <v>sla</v>
+      </c>
+      <c r="D42" t="str">
+        <v/>
+      </c>
+      <c r="E42" t="str">
+        <v/>
+      </c>
+      <c r="F42" t="str">
+        <v/>
+      </c>
+      <c r="G42" t="str">
+        <v/>
+      </c>
+      <c r="H42" t="str">
+        <v/>
+      </c>
+      <c r="I42" t="str">
+        <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>paddenstoelen</v>
+        <v>jalapenos</v>
       </c>
       <c r="B43" t="str">
-        <v>champignons</v>
+        <v>jalapeño</v>
+      </c>
+      <c r="C43" t="str">
+        <v/>
+      </c>
+      <c r="D43" t="str">
+        <v/>
+      </c>
+      <c r="E43" t="str">
+        <v/>
+      </c>
+      <c r="F43" t="str">
+        <v/>
+      </c>
+      <c r="G43" t="str">
+        <v/>
+      </c>
+      <c r="H43" t="str">
+        <v/>
+      </c>
+      <c r="I43" t="str">
+        <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>chili</v>
+        <v>kalkoenlapjes</v>
       </c>
       <c r="B44" t="str">
-        <v>chilipepers</v>
+        <v>kalkoen</v>
+      </c>
+      <c r="C44" t="str">
+        <v/>
+      </c>
+      <c r="D44" t="str">
+        <v/>
+      </c>
+      <c r="E44" t="str">
+        <v/>
+      </c>
+      <c r="F44" t="str">
+        <v/>
+      </c>
+      <c r="G44" t="str">
+        <v/>
+      </c>
+      <c r="H44" t="str">
+        <v/>
+      </c>
+      <c r="I44" t="str">
+        <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>chilivlokken</v>
+        <v>kerstomaatjes</v>
       </c>
       <c r="B45" t="str">
-        <v>chilipepers</v>
+        <v>cherry tomaten</v>
+      </c>
+      <c r="C45" t="str">
+        <v>cherrytomaatje</v>
+      </c>
+      <c r="D45" t="str">
+        <v>cherrytomaatjes</v>
+      </c>
+      <c r="E45" t="str">
+        <v>kerstomaat</v>
+      </c>
+      <c r="F45" t="str">
+        <v>kerstomaten</v>
+      </c>
+      <c r="G45" t="str">
+        <v/>
+      </c>
+      <c r="H45" t="str">
+        <v/>
+      </c>
+      <c r="I45" t="str">
+        <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>rode peper</v>
+        <v>kipdijfilet</v>
       </c>
       <c r="B46" t="str">
-        <v>chilipepers</v>
+        <v>kipdij</v>
+      </c>
+      <c r="C46" t="str">
+        <v>kipdijen</v>
+      </c>
+      <c r="D46" t="str">
+        <v>kippenboutenfilet</v>
+      </c>
+      <c r="E46" t="str">
+        <v>kippendijen</v>
+      </c>
+      <c r="F46" t="str">
+        <v>kippendijenfilet</v>
+      </c>
+      <c r="G46" t="str">
+        <v/>
+      </c>
+      <c r="H46" t="str">
+        <v/>
+      </c>
+      <c r="I46" t="str">
+        <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>melkchocolade</v>
+        <v>kipfilet</v>
       </c>
       <c r="B47" t="str">
-        <v>chocolade</v>
+        <v>kip</v>
+      </c>
+      <c r="C47" t="str">
+        <v>kippenborst</v>
+      </c>
+      <c r="D47" t="str">
+        <v/>
+      </c>
+      <c r="E47" t="str">
+        <v/>
+      </c>
+      <c r="F47" t="str">
+        <v/>
+      </c>
+      <c r="G47" t="str">
+        <v/>
+      </c>
+      <c r="H47" t="str">
+        <v/>
+      </c>
+      <c r="I47" t="str">
+        <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>pure chocolade</v>
+        <v>kippenbouillon</v>
       </c>
       <c r="B48" t="str">
-        <v>chocolade</v>
+        <v>kippenbouillon</v>
+      </c>
+      <c r="C48" t="str">
+        <v/>
+      </c>
+      <c r="D48" t="str">
+        <v/>
+      </c>
+      <c r="E48" t="str">
+        <v/>
+      </c>
+      <c r="F48" t="str">
+        <v/>
+      </c>
+      <c r="G48" t="str">
+        <v/>
+      </c>
+      <c r="H48" t="str">
+        <v/>
+      </c>
+      <c r="I48" t="str">
+        <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>citroensap</v>
+        <v>kippenkruiden</v>
       </c>
       <c r="B49" t="str">
-        <v>citroen</v>
+        <v>bbq kruiden</v>
+      </c>
+      <c r="C49" t="str">
+        <v>kippenkruiden</v>
+      </c>
+      <c r="D49" t="str">
+        <v/>
+      </c>
+      <c r="E49" t="str">
+        <v/>
+      </c>
+      <c r="F49" t="str">
+        <v/>
+      </c>
+      <c r="G49" t="str">
+        <v/>
+      </c>
+      <c r="H49" t="str">
+        <v/>
+      </c>
+      <c r="I49" t="str">
+        <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>currypoeder</v>
+        <v>kippenworsten</v>
       </c>
       <c r="B50" t="str">
-        <v>curry</v>
+        <v>kippenworst</v>
+      </c>
+      <c r="C50" t="str">
+        <v/>
+      </c>
+      <c r="D50" t="str">
+        <v/>
+      </c>
+      <c r="E50" t="str">
+        <v/>
+      </c>
+      <c r="F50" t="str">
+        <v/>
+      </c>
+      <c r="G50" t="str">
+        <v/>
+      </c>
+      <c r="H50" t="str">
+        <v/>
+      </c>
+      <c r="I50" t="str">
+        <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>ei</v>
+        <v>kipschnitzel</v>
       </c>
       <c r="B51" t="str">
-        <v>eieren_1</v>
+        <v>kippenschnitzel</v>
+      </c>
+      <c r="C51" t="str">
+        <v/>
+      </c>
+      <c r="D51" t="str">
+        <v/>
+      </c>
+      <c r="E51" t="str">
+        <v/>
+      </c>
+      <c r="F51" t="str">
+        <v/>
+      </c>
+      <c r="G51" t="str">
+        <v/>
+      </c>
+      <c r="H51" t="str">
+        <v/>
+      </c>
+      <c r="I51" t="str">
+        <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>eieren</v>
+        <v>kokosmelk</v>
       </c>
       <c r="B52" t="str">
-        <v>eieren_1</v>
+        <v>kokosmelk</v>
+      </c>
+      <c r="C52" t="str">
+        <v>kokosroom</v>
+      </c>
+      <c r="D52" t="str">
+        <v/>
+      </c>
+      <c r="E52" t="str">
+        <v/>
+      </c>
+      <c r="F52" t="str">
+        <v/>
+      </c>
+      <c r="G52" t="str">
+        <v/>
+      </c>
+      <c r="H52" t="str">
+        <v/>
+      </c>
+      <c r="I52" t="str">
+        <v/>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>framboos</v>
+        <v>kokosolie</v>
       </c>
       <c r="B53" t="str">
-        <v>frambozen</v>
+        <v>kokosolie</v>
+      </c>
+      <c r="C53" t="str">
+        <v>kokosvet</v>
+      </c>
+      <c r="D53" t="str">
+        <v/>
+      </c>
+      <c r="E53" t="str">
+        <v/>
+      </c>
+      <c r="F53" t="str">
+        <v/>
+      </c>
+      <c r="G53" t="str">
+        <v/>
+      </c>
+      <c r="H53" t="str">
+        <v/>
+      </c>
+      <c r="I53" t="str">
+        <v/>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>droge gist</v>
+        <v>komkommer</v>
       </c>
       <c r="B54" t="str">
-        <v>gedroogde_gist</v>
+        <v>komkommertje</v>
+      </c>
+      <c r="C54" t="str">
+        <v/>
+      </c>
+      <c r="D54" t="str">
+        <v/>
+      </c>
+      <c r="E54" t="str">
+        <v/>
+      </c>
+      <c r="F54" t="str">
+        <v/>
+      </c>
+      <c r="G54" t="str">
+        <v/>
+      </c>
+      <c r="H54" t="str">
+        <v/>
+      </c>
+      <c r="I54" t="str">
+        <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>droogzout</v>
+        <v>koriander</v>
       </c>
       <c r="B55" t="str">
-        <v>gedroogde_gist</v>
+        <v>verse koriander</v>
+      </c>
+      <c r="C55" t="str">
+        <v/>
+      </c>
+      <c r="D55" t="str">
+        <v/>
+      </c>
+      <c r="E55" t="str">
+        <v/>
+      </c>
+      <c r="F55" t="str">
+        <v/>
+      </c>
+      <c r="G55" t="str">
+        <v/>
+      </c>
+      <c r="H55" t="str">
+        <v/>
+      </c>
+      <c r="I55" t="str">
+        <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>gehakt vlees</v>
+        <v>lasagnevellen</v>
       </c>
       <c r="B56" t="str">
-        <v>gehakt</v>
+        <v>pasta</v>
+      </c>
+      <c r="C56" t="str">
+        <v/>
+      </c>
+      <c r="D56" t="str">
+        <v/>
+      </c>
+      <c r="E56" t="str">
+        <v/>
+      </c>
+      <c r="F56" t="str">
+        <v/>
+      </c>
+      <c r="G56" t="str">
+        <v/>
+      </c>
+      <c r="H56" t="str">
+        <v/>
+      </c>
+      <c r="I56" t="str">
+        <v/>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>rundergehakt</v>
+        <v>laurier</v>
       </c>
       <c r="B57" t="str">
-        <v>gehakt</v>
+        <v>laurierblaadjes</v>
+      </c>
+      <c r="C57" t="str">
+        <v>laurierblad</v>
+      </c>
+      <c r="D57" t="str">
+        <v/>
+      </c>
+      <c r="E57" t="str">
+        <v/>
+      </c>
+      <c r="F57" t="str">
+        <v/>
+      </c>
+      <c r="G57" t="str">
+        <v/>
+      </c>
+      <c r="H57" t="str">
+        <v/>
+      </c>
+      <c r="I57" t="str">
+        <v/>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>varkensgehakt</v>
+        <v>limoen</v>
       </c>
       <c r="B58" t="str">
-        <v>gehakt</v>
+        <v>limoen</v>
+      </c>
+      <c r="C58" t="str">
+        <v>limoensap</v>
+      </c>
+      <c r="D58" t="str">
+        <v/>
+      </c>
+      <c r="E58" t="str">
+        <v/>
+      </c>
+      <c r="F58" t="str">
+        <v/>
+      </c>
+      <c r="G58" t="str">
+        <v/>
+      </c>
+      <c r="H58" t="str">
+        <v/>
+      </c>
+      <c r="I58" t="str">
+        <v/>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>gehakte noten</v>
+        <v>look</v>
       </c>
       <c r="B59" t="str">
-        <v>gehakte_walnoten</v>
+        <v>knoflook</v>
+      </c>
+      <c r="C59" t="str">
+        <v>knoflookteentje</v>
+      </c>
+      <c r="D59" t="str">
+        <v>knoflookteentjes</v>
+      </c>
+      <c r="E59" t="str">
+        <v>lookteentje</v>
+      </c>
+      <c r="F59" t="str">
+        <v>lookteentjes</v>
+      </c>
+      <c r="G59" t="str">
+        <v>teentje knoflook</v>
+      </c>
+      <c r="H59" t="str">
+        <v>teentjes knoflook</v>
+      </c>
+      <c r="I59" t="str">
+        <v/>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>gele paprika</v>
+        <v>mais</v>
       </c>
       <c r="B60" t="str">
-        <v>gele_paprika</v>
+        <v>mais</v>
+      </c>
+      <c r="C60" t="str">
+        <v>maïs</v>
+      </c>
+      <c r="D60" t="str">
+        <v>maiskorrels</v>
+      </c>
+      <c r="E60" t="str">
+        <v>maïskorrels</v>
+      </c>
+      <c r="F60" t="str">
+        <v/>
+      </c>
+      <c r="G60" t="str">
+        <v/>
+      </c>
+      <c r="H60" t="str">
+        <v/>
+      </c>
+      <c r="I60" t="str">
+        <v/>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>gemberpowder</v>
+        <v>maizena</v>
       </c>
       <c r="B61" t="str">
-        <v>gember</v>
+        <v>maïzena</v>
+      </c>
+      <c r="C61" t="str">
+        <v>zetmeel</v>
+      </c>
+      <c r="D61" t="str">
+        <v/>
+      </c>
+      <c r="E61" t="str">
+        <v/>
+      </c>
+      <c r="F61" t="str">
+        <v/>
+      </c>
+      <c r="G61" t="str">
+        <v/>
+      </c>
+      <c r="H61" t="str">
+        <v/>
+      </c>
+      <c r="I61" t="str">
+        <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>verse gember</v>
+        <v>mandarijnen</v>
       </c>
       <c r="B62" t="str">
-        <v>gember</v>
+        <v>mandarijn</v>
+      </c>
+      <c r="C62" t="str">
+        <v/>
+      </c>
+      <c r="D62" t="str">
+        <v/>
+      </c>
+      <c r="E62" t="str">
+        <v/>
+      </c>
+      <c r="F62" t="str">
+        <v/>
+      </c>
+      <c r="G62" t="str">
+        <v/>
+      </c>
+      <c r="H62" t="str">
+        <v/>
+      </c>
+      <c r="I62" t="str">
+        <v/>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>geraspte kaas</v>
+        <v>mayonaise</v>
       </c>
       <c r="B63" t="str">
-        <v>geraspte_kaas</v>
+        <v>mayonnaise</v>
+      </c>
+      <c r="C63" t="str">
+        <v/>
+      </c>
+      <c r="D63" t="str">
+        <v/>
+      </c>
+      <c r="E63" t="str">
+        <v/>
+      </c>
+      <c r="F63" t="str">
+        <v/>
+      </c>
+      <c r="G63" t="str">
+        <v/>
+      </c>
+      <c r="H63" t="str">
+        <v/>
+      </c>
+      <c r="I63" t="str">
+        <v/>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>gruyere</v>
+        <v>melk</v>
       </c>
       <c r="B64" t="str">
-        <v>geraspte_kaas</v>
+        <v>halfvolle melk</v>
+      </c>
+      <c r="C64" t="str">
+        <v>volle melk</v>
+      </c>
+      <c r="D64" t="str">
+        <v/>
+      </c>
+      <c r="E64" t="str">
+        <v/>
+      </c>
+      <c r="F64" t="str">
+        <v/>
+      </c>
+      <c r="G64" t="str">
+        <v/>
+      </c>
+      <c r="H64" t="str">
+        <v/>
+      </c>
+      <c r="I64" t="str">
+        <v/>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>gruyère</v>
+        <v>mini_komkommers</v>
       </c>
       <c r="B65" t="str">
-        <v>geraspte_kaas</v>
+        <v>mini komkommer</v>
+      </c>
+      <c r="C65" t="str">
+        <v>mini komkommers</v>
+      </c>
+      <c r="D65" t="str">
+        <v/>
+      </c>
+      <c r="E65" t="str">
+        <v/>
+      </c>
+      <c r="F65" t="str">
+        <v/>
+      </c>
+      <c r="G65" t="str">
+        <v/>
+      </c>
+      <c r="H65" t="str">
+        <v/>
+      </c>
+      <c r="I65" t="str">
+        <v/>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>kaas</v>
+        <v>mosterd</v>
       </c>
       <c r="B66" t="str">
-        <v>geraspte_kaas</v>
+        <v>dijonmmosterd</v>
+      </c>
+      <c r="C66" t="str">
+        <v>mosterd</v>
+      </c>
+      <c r="D66" t="str">
+        <v/>
+      </c>
+      <c r="E66" t="str">
+        <v/>
+      </c>
+      <c r="F66" t="str">
+        <v/>
+      </c>
+      <c r="G66" t="str">
+        <v/>
+      </c>
+      <c r="H66" t="str">
+        <v/>
+      </c>
+      <c r="I66" t="str">
+        <v/>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>geraspte wortel</v>
+        <v>mozarella</v>
       </c>
       <c r="B67" t="str">
-        <v>geraspte_wortelen</v>
+        <v>mozzarella</v>
+      </c>
+      <c r="C67" t="str">
+        <v>mozzarelle</v>
+      </c>
+      <c r="D67" t="str">
+        <v/>
+      </c>
+      <c r="E67" t="str">
+        <v/>
+      </c>
+      <c r="F67" t="str">
+        <v/>
+      </c>
+      <c r="G67" t="str">
+        <v/>
+      </c>
+      <c r="H67" t="str">
+        <v/>
+      </c>
+      <c r="I67" t="str">
+        <v/>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>geraspte wortels</v>
+        <v>munt</v>
       </c>
       <c r="B68" t="str">
-        <v>geraspte_wortelen</v>
+        <v>verse munt</v>
+      </c>
+      <c r="C68" t="str">
+        <v/>
+      </c>
+      <c r="D68" t="str">
+        <v/>
+      </c>
+      <c r="E68" t="str">
+        <v/>
+      </c>
+      <c r="F68" t="str">
+        <v/>
+      </c>
+      <c r="G68" t="str">
+        <v/>
+      </c>
+      <c r="H68" t="str">
+        <v/>
+      </c>
+      <c r="I68" t="str">
+        <v/>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>gerookte zalm</v>
+        <v>olijfolie</v>
       </c>
       <c r="B69" t="str">
-        <v>gerookte_zalm</v>
+        <v>extra vergine olijfolie</v>
+      </c>
+      <c r="C69" t="str">
+        <v>olijfolie extra vierge</v>
+      </c>
+      <c r="D69" t="str">
+        <v/>
+      </c>
+      <c r="E69" t="str">
+        <v/>
+      </c>
+      <c r="F69" t="str">
+        <v/>
+      </c>
+      <c r="G69" t="str">
+        <v/>
+      </c>
+      <c r="H69" t="str">
+        <v/>
+      </c>
+      <c r="I69" t="str">
+        <v/>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>geklaarde boter</v>
+        <v>paksoi</v>
       </c>
       <c r="B70" t="str">
-        <v>ghee</v>
+        <v>paksoy</v>
+      </c>
+      <c r="C70" t="str">
+        <v/>
+      </c>
+      <c r="D70" t="str">
+        <v/>
+      </c>
+      <c r="E70" t="str">
+        <v/>
+      </c>
+      <c r="F70" t="str">
+        <v/>
+      </c>
+      <c r="G70" t="str">
+        <v/>
+      </c>
+      <c r="H70" t="str">
+        <v/>
+      </c>
+      <c r="I70" t="str">
+        <v/>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>ghee</v>
+        <v>paneermeel</v>
       </c>
       <c r="B71" t="str">
-        <v>ghee</v>
+        <v>broodkruim</v>
+      </c>
+      <c r="C71" t="str">
+        <v>broodkruimels</v>
+      </c>
+      <c r="D71" t="str">
+        <v/>
+      </c>
+      <c r="E71" t="str">
+        <v/>
+      </c>
+      <c r="F71" t="str">
+        <v/>
+      </c>
+      <c r="G71" t="str">
+        <v/>
+      </c>
+      <c r="H71" t="str">
+        <v/>
+      </c>
+      <c r="I71" t="str">
+        <v/>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>asperge</v>
+        <v>paprika</v>
       </c>
       <c r="B72" t="str">
-        <v>groene_asperges</v>
+        <v>groene paprika</v>
+      </c>
+      <c r="C72" t="str">
+        <v>paprika</v>
+      </c>
+      <c r="D72" t="str">
+        <v>rode paprika</v>
+      </c>
+      <c r="E72" t="str">
+        <v/>
+      </c>
+      <c r="F72" t="str">
+        <v/>
+      </c>
+      <c r="G72" t="str">
+        <v/>
+      </c>
+      <c r="H72" t="str">
+        <v/>
+      </c>
+      <c r="I72" t="str">
+        <v/>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>asperges</v>
+        <v>parmaham</v>
       </c>
       <c r="B73" t="str">
-        <v>groene_asperges</v>
+        <v>parma ham</v>
+      </c>
+      <c r="C73" t="str">
+        <v>rauwe ham</v>
+      </c>
+      <c r="D73" t="str">
+        <v/>
+      </c>
+      <c r="E73" t="str">
+        <v/>
+      </c>
+      <c r="F73" t="str">
+        <v/>
+      </c>
+      <c r="G73" t="str">
+        <v/>
+      </c>
+      <c r="H73" t="str">
+        <v/>
+      </c>
+      <c r="I73" t="str">
+        <v/>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>groentenbouillon</v>
+        <v>parmezaan</v>
       </c>
       <c r="B74" t="str">
-        <v>groentenbouillon</v>
+        <v>parmezaan kaas</v>
+      </c>
+      <c r="C74" t="str">
+        <v>parmezaankaas</v>
+      </c>
+      <c r="D74" t="str">
+        <v>parmezaanse kaas</v>
+      </c>
+      <c r="E74" t="str">
+        <v/>
+      </c>
+      <c r="F74" t="str">
+        <v/>
+      </c>
+      <c r="G74" t="str">
+        <v/>
+      </c>
+      <c r="H74" t="str">
+        <v/>
+      </c>
+      <c r="I74" t="str">
+        <v/>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>hagelslag</v>
+        <v>passata</v>
       </c>
       <c r="B75" t="str">
-        <v>hagelslag</v>
+        <v>passata</v>
+      </c>
+      <c r="C75" t="str">
+        <v/>
+      </c>
+      <c r="D75" t="str">
+        <v/>
+      </c>
+      <c r="E75" t="str">
+        <v/>
+      </c>
+      <c r="F75" t="str">
+        <v/>
+      </c>
+      <c r="G75" t="str">
+        <v/>
+      </c>
+      <c r="H75" t="str">
+        <v/>
+      </c>
+      <c r="I75" t="str">
+        <v/>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>hazelnoot</v>
+        <v>peren</v>
       </c>
       <c r="B76" t="str">
-        <v>hazelnoten</v>
+        <v>peer</v>
+      </c>
+      <c r="C76" t="str">
+        <v/>
+      </c>
+      <c r="D76" t="str">
+        <v/>
+      </c>
+      <c r="E76" t="str">
+        <v/>
+      </c>
+      <c r="F76" t="str">
+        <v/>
+      </c>
+      <c r="G76" t="str">
+        <v/>
+      </c>
+      <c r="H76" t="str">
+        <v/>
+      </c>
+      <c r="I76" t="str">
+        <v/>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>honing</v>
+        <v>peterselie</v>
       </c>
       <c r="B77" t="str">
-        <v>honing</v>
+        <v>verse peterselie</v>
+      </c>
+      <c r="C77" t="str">
+        <v/>
+      </c>
+      <c r="D77" t="str">
+        <v/>
+      </c>
+      <c r="E77" t="str">
+        <v/>
+      </c>
+      <c r="F77" t="str">
+        <v/>
+      </c>
+      <c r="G77" t="str">
+        <v/>
+      </c>
+      <c r="H77" t="str">
+        <v/>
+      </c>
+      <c r="I77" t="str">
+        <v/>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>vloeibare honing</v>
+        <v>pijpajuin</v>
       </c>
       <c r="B78" t="str">
-        <v>honing</v>
+        <v>bosui</v>
+      </c>
+      <c r="C78" t="str">
+        <v>bosuitje</v>
+      </c>
+      <c r="D78" t="str">
+        <v>bosuitjes</v>
+      </c>
+      <c r="E78" t="str">
+        <v>lente-ui</v>
+      </c>
+      <c r="F78" t="str">
+        <v>lenteui</v>
+      </c>
+      <c r="G78" t="str">
+        <v>lenteuitje</v>
+      </c>
+      <c r="H78" t="str">
+        <v>pijpajuintje</v>
+      </c>
+      <c r="I78" t="str">
+        <v/>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>ijssla</v>
+        <v>platte_kaas</v>
       </c>
       <c r="B79" t="str">
-        <v>ijsbergsla</v>
+        <v>kwark</v>
+      </c>
+      <c r="C79" t="str">
+        <v>platte kaas</v>
+      </c>
+      <c r="D79" t="str">
+        <v/>
+      </c>
+      <c r="E79" t="str">
+        <v/>
+      </c>
+      <c r="F79" t="str">
+        <v/>
+      </c>
+      <c r="G79" t="str">
+        <v/>
+      </c>
+      <c r="H79" t="str">
+        <v/>
+      </c>
+      <c r="I79" t="str">
+        <v/>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>sla</v>
+        <v>pudding_poeder</v>
       </c>
       <c r="B80" t="str">
-        <v>ijsbergsla</v>
+        <v>pudding</v>
+      </c>
+      <c r="C80" t="str">
+        <v>puddingpoeder</v>
+      </c>
+      <c r="D80" t="str">
+        <v/>
+      </c>
+      <c r="E80" t="str">
+        <v/>
+      </c>
+      <c r="F80" t="str">
+        <v/>
+      </c>
+      <c r="G80" t="str">
+        <v/>
+      </c>
+      <c r="H80" t="str">
+        <v/>
+      </c>
+      <c r="I80" t="str">
+        <v/>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>jalapeño</v>
+        <v>radijsjes</v>
       </c>
       <c r="B81" t="str">
-        <v>jalapenos</v>
+        <v>radijs</v>
+      </c>
+      <c r="C81" t="str">
+        <v>radiJs</v>
+      </c>
+      <c r="D81" t="str">
+        <v/>
+      </c>
+      <c r="E81" t="str">
+        <v/>
+      </c>
+      <c r="F81" t="str">
+        <v/>
+      </c>
+      <c r="G81" t="str">
+        <v/>
+      </c>
+      <c r="H81" t="str">
+        <v/>
+      </c>
+      <c r="I81" t="str">
+        <v/>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>kalkoen</v>
+        <v>rijstpapier</v>
       </c>
       <c r="B82" t="str">
-        <v>kalkoenlapjes</v>
+        <v>rijstvellen</v>
+      </c>
+      <c r="C82" t="str">
+        <v/>
+      </c>
+      <c r="D82" t="str">
+        <v/>
+      </c>
+      <c r="E82" t="str">
+        <v/>
+      </c>
+      <c r="F82" t="str">
+        <v/>
+      </c>
+      <c r="G82" t="str">
+        <v/>
+      </c>
+      <c r="H82" t="str">
+        <v/>
+      </c>
+      <c r="I82" t="str">
+        <v/>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>cherry tomaten</v>
+        <v>rode_ajuin</v>
       </c>
       <c r="B83" t="str">
-        <v>kerstomaatjes</v>
+        <v>rode ajuin</v>
+      </c>
+      <c r="C83" t="str">
+        <v>rode ui</v>
+      </c>
+      <c r="D83" t="str">
+        <v>rode uien</v>
+      </c>
+      <c r="E83" t="str">
+        <v/>
+      </c>
+      <c r="F83" t="str">
+        <v/>
+      </c>
+      <c r="G83" t="str">
+        <v/>
+      </c>
+      <c r="H83" t="str">
+        <v/>
+      </c>
+      <c r="I83" t="str">
+        <v/>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>cherrytomaatje</v>
+        <v>rode_currypasta</v>
       </c>
       <c r="B84" t="str">
-        <v>kerstomaatjes</v>
+        <v>currypasta</v>
+      </c>
+      <c r="C84" t="str">
+        <v/>
+      </c>
+      <c r="D84" t="str">
+        <v/>
+      </c>
+      <c r="E84" t="str">
+        <v/>
+      </c>
+      <c r="F84" t="str">
+        <v/>
+      </c>
+      <c r="G84" t="str">
+        <v/>
+      </c>
+      <c r="H84" t="str">
+        <v/>
+      </c>
+      <c r="I84" t="str">
+        <v/>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>cherrytomaatjes</v>
+        <v>rode_wijn</v>
       </c>
       <c r="B85" t="str">
-        <v>kerstomaatjes</v>
+        <v>rode wijn</v>
+      </c>
+      <c r="C85" t="str">
+        <v/>
+      </c>
+      <c r="D85" t="str">
+        <v/>
+      </c>
+      <c r="E85" t="str">
+        <v/>
+      </c>
+      <c r="F85" t="str">
+        <v/>
+      </c>
+      <c r="G85" t="str">
+        <v/>
+      </c>
+      <c r="H85" t="str">
+        <v/>
+      </c>
+      <c r="I85" t="str">
+        <v/>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>kerstomaat</v>
+        <v>room</v>
       </c>
       <c r="B86" t="str">
-        <v>kerstomaatjes</v>
+        <v>room</v>
+      </c>
+      <c r="C86" t="str">
+        <v>slagroom</v>
+      </c>
+      <c r="D86" t="str">
+        <v/>
+      </c>
+      <c r="E86" t="str">
+        <v/>
+      </c>
+      <c r="F86" t="str">
+        <v/>
+      </c>
+      <c r="G86" t="str">
+        <v/>
+      </c>
+      <c r="H86" t="str">
+        <v/>
+      </c>
+      <c r="I86" t="str">
+        <v/>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>kerstomaten</v>
+        <v>rozemarijn</v>
       </c>
       <c r="B87" t="str">
-        <v>kerstomaatjes</v>
+        <v>verse rozemarijn</v>
+      </c>
+      <c r="C87" t="str">
+        <v/>
+      </c>
+      <c r="D87" t="str">
+        <v/>
+      </c>
+      <c r="E87" t="str">
+        <v/>
+      </c>
+      <c r="F87" t="str">
+        <v/>
+      </c>
+      <c r="G87" t="str">
+        <v/>
+      </c>
+      <c r="H87" t="str">
+        <v/>
+      </c>
+      <c r="I87" t="str">
+        <v/>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>kipdij</v>
+        <v>rundsbouillon</v>
       </c>
       <c r="B88" t="str">
-        <v>kipdijfilet</v>
+        <v>runderbouillon</v>
+      </c>
+      <c r="C88" t="str">
+        <v/>
+      </c>
+      <c r="D88" t="str">
+        <v/>
+      </c>
+      <c r="E88" t="str">
+        <v/>
+      </c>
+      <c r="F88" t="str">
+        <v/>
+      </c>
+      <c r="G88" t="str">
+        <v/>
+      </c>
+      <c r="H88" t="str">
+        <v/>
+      </c>
+      <c r="I88" t="str">
+        <v/>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>kipdijen</v>
+        <v>satekruiden</v>
       </c>
       <c r="B89" t="str">
-        <v>kipdijfilet</v>
+        <v>satékruiden</v>
+      </c>
+      <c r="C89" t="str">
+        <v>satésaus</v>
+      </c>
+      <c r="D89" t="str">
+        <v/>
+      </c>
+      <c r="E89" t="str">
+        <v/>
+      </c>
+      <c r="F89" t="str">
+        <v/>
+      </c>
+      <c r="G89" t="str">
+        <v/>
+      </c>
+      <c r="H89" t="str">
+        <v/>
+      </c>
+      <c r="I89" t="str">
+        <v/>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>kippenboutenfilet</v>
+        <v>scampis</v>
       </c>
       <c r="B90" t="str">
-        <v>kipdijfilet</v>
+        <v>oester</v>
+      </c>
+      <c r="C90" t="str">
+        <v>scampi</v>
+      </c>
+      <c r="D90" t="str">
+        <v/>
+      </c>
+      <c r="E90" t="str">
+        <v/>
+      </c>
+      <c r="F90" t="str">
+        <v/>
+      </c>
+      <c r="G90" t="str">
+        <v/>
+      </c>
+      <c r="H90" t="str">
+        <v/>
+      </c>
+      <c r="I90" t="str">
+        <v/>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>kippendijen</v>
+        <v>selder</v>
       </c>
       <c r="B91" t="str">
-        <v>kipdijfilet</v>
+        <v>selderie</v>
+      </c>
+      <c r="C91" t="str">
+        <v>selderij</v>
+      </c>
+      <c r="D91" t="str">
+        <v/>
+      </c>
+      <c r="E91" t="str">
+        <v/>
+      </c>
+      <c r="F91" t="str">
+        <v/>
+      </c>
+      <c r="G91" t="str">
+        <v/>
+      </c>
+      <c r="H91" t="str">
+        <v/>
+      </c>
+      <c r="I91" t="str">
+        <v/>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>kippendijenfilet</v>
+        <v>sesamolie</v>
       </c>
       <c r="B92" t="str">
-        <v>kipdijfilet</v>
+        <v>sesamolie</v>
+      </c>
+      <c r="C92" t="str">
+        <v/>
+      </c>
+      <c r="D92" t="str">
+        <v/>
+      </c>
+      <c r="E92" t="str">
+        <v/>
+      </c>
+      <c r="F92" t="str">
+        <v/>
+      </c>
+      <c r="G92" t="str">
+        <v/>
+      </c>
+      <c r="H92" t="str">
+        <v/>
+      </c>
+      <c r="I92" t="str">
+        <v/>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>kip</v>
+        <v>sjalotten</v>
       </c>
       <c r="B93" t="str">
-        <v>kipfilet</v>
+        <v>sjalot</v>
+      </c>
+      <c r="C93" t="str">
+        <v>sjalotje</v>
+      </c>
+      <c r="D93" t="str">
+        <v>sjalotjes</v>
+      </c>
+      <c r="E93" t="str">
+        <v/>
+      </c>
+      <c r="F93" t="str">
+        <v/>
+      </c>
+      <c r="G93" t="str">
+        <v/>
+      </c>
+      <c r="H93" t="str">
+        <v/>
+      </c>
+      <c r="I93" t="str">
+        <v/>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>kippenborst</v>
+        <v>sojasaus</v>
       </c>
       <c r="B94" t="str">
-        <v>kipfilet</v>
+        <v>soja saus</v>
+      </c>
+      <c r="C94" t="str">
+        <v>sojasaus</v>
+      </c>
+      <c r="D94" t="str">
+        <v/>
+      </c>
+      <c r="E94" t="str">
+        <v/>
+      </c>
+      <c r="F94" t="str">
+        <v/>
+      </c>
+      <c r="G94" t="str">
+        <v/>
+      </c>
+      <c r="H94" t="str">
+        <v/>
+      </c>
+      <c r="I94" t="str">
+        <v/>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>kippenbouillon</v>
+        <v>spekblokjes</v>
       </c>
       <c r="B95" t="str">
-        <v>kippenbouillon</v>
+        <v>lardons</v>
+      </c>
+      <c r="C95" t="str">
+        <v>spekblokje</v>
+      </c>
+      <c r="D95" t="str">
+        <v/>
+      </c>
+      <c r="E95" t="str">
+        <v/>
+      </c>
+      <c r="F95" t="str">
+        <v/>
+      </c>
+      <c r="G95" t="str">
+        <v/>
+      </c>
+      <c r="H95" t="str">
+        <v/>
+      </c>
+      <c r="I95" t="str">
+        <v/>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>bbq kruiden</v>
+        <v>speltbloem</v>
       </c>
       <c r="B96" t="str">
-        <v>kippenkruiden</v>
+        <v>speltmeel</v>
+      </c>
+      <c r="C96" t="str">
+        <v/>
+      </c>
+      <c r="D96" t="str">
+        <v/>
+      </c>
+      <c r="E96" t="str">
+        <v/>
+      </c>
+      <c r="F96" t="str">
+        <v/>
+      </c>
+      <c r="G96" t="str">
+        <v/>
+      </c>
+      <c r="H96" t="str">
+        <v/>
+      </c>
+      <c r="I96" t="str">
+        <v/>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>kippenkruiden</v>
+        <v>suiker</v>
       </c>
       <c r="B97" t="str">
-        <v>kippenkruiden</v>
+        <v>fijne suiker</v>
+      </c>
+      <c r="C97" t="str">
+        <v>kristalsuiker</v>
+      </c>
+      <c r="D97" t="str">
+        <v/>
+      </c>
+      <c r="E97" t="str">
+        <v/>
+      </c>
+      <c r="F97" t="str">
+        <v/>
+      </c>
+      <c r="G97" t="str">
+        <v/>
+      </c>
+      <c r="H97" t="str">
+        <v/>
+      </c>
+      <c r="I97" t="str">
+        <v/>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>kippenworst</v>
+        <v>suikerklontjes</v>
       </c>
       <c r="B98" t="str">
-        <v>kippenworsten</v>
+        <v>suikerklontje</v>
+      </c>
+      <c r="C98" t="str">
+        <v/>
+      </c>
+      <c r="D98" t="str">
+        <v/>
+      </c>
+      <c r="E98" t="str">
+        <v/>
+      </c>
+      <c r="F98" t="str">
+        <v/>
+      </c>
+      <c r="G98" t="str">
+        <v/>
+      </c>
+      <c r="H98" t="str">
+        <v/>
+      </c>
+      <c r="I98" t="str">
+        <v/>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>kippenschnitzel</v>
+        <v>tijm</v>
       </c>
       <c r="B99" t="str">
-        <v>kipschnitzel</v>
+        <v>verse tijm</v>
+      </c>
+      <c r="C99" t="str">
+        <v/>
+      </c>
+      <c r="D99" t="str">
+        <v/>
+      </c>
+      <c r="E99" t="str">
+        <v/>
+      </c>
+      <c r="F99" t="str">
+        <v/>
+      </c>
+      <c r="G99" t="str">
+        <v/>
+      </c>
+      <c r="H99" t="str">
+        <v/>
+      </c>
+      <c r="I99" t="str">
+        <v/>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>kokosmelk</v>
+        <v>tomaten</v>
       </c>
       <c r="B100" t="str">
-        <v>kokosmelk</v>
+        <v>tomaat</v>
+      </c>
+      <c r="C100" t="str">
+        <v>tomaatje</v>
+      </c>
+      <c r="D100" t="str">
+        <v/>
+      </c>
+      <c r="E100" t="str">
+        <v/>
+      </c>
+      <c r="F100" t="str">
+        <v/>
+      </c>
+      <c r="G100" t="str">
+        <v/>
+      </c>
+      <c r="H100" t="str">
+        <v/>
+      </c>
+      <c r="I100" t="str">
+        <v/>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>kokosroom</v>
+        <v>tomaten_uit_blik</v>
       </c>
       <c r="B101" t="str">
-        <v>kokosmelk</v>
+        <v>tomaten uit blik</v>
+      </c>
+      <c r="C101" t="str">
+        <v/>
+      </c>
+      <c r="D101" t="str">
+        <v/>
+      </c>
+      <c r="E101" t="str">
+        <v/>
+      </c>
+      <c r="F101" t="str">
+        <v/>
+      </c>
+      <c r="G101" t="str">
+        <v/>
+      </c>
+      <c r="H101" t="str">
+        <v/>
+      </c>
+      <c r="I101" t="str">
+        <v/>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>kokosolie</v>
+        <v>tomatenblokjes</v>
       </c>
       <c r="B102" t="str">
-        <v>kokosolie</v>
+        <v>tomatenblokjes</v>
+      </c>
+      <c r="C102" t="str">
+        <v/>
+      </c>
+      <c r="D102" t="str">
+        <v/>
+      </c>
+      <c r="E102" t="str">
+        <v/>
+      </c>
+      <c r="F102" t="str">
+        <v/>
+      </c>
+      <c r="G102" t="str">
+        <v/>
+      </c>
+      <c r="H102" t="str">
+        <v/>
+      </c>
+      <c r="I102" t="str">
+        <v/>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>kokosvet</v>
+        <v>tomatenpuree</v>
       </c>
       <c r="B103" t="str">
-        <v>kokosolie</v>
+        <v>geconcentreerde tomatenpuree</v>
+      </c>
+      <c r="C103" t="str">
+        <v>tomatenpuree</v>
+      </c>
+      <c r="D103" t="str">
+        <v/>
+      </c>
+      <c r="E103" t="str">
+        <v/>
+      </c>
+      <c r="F103" t="str">
+        <v/>
+      </c>
+      <c r="G103" t="str">
+        <v/>
+      </c>
+      <c r="H103" t="str">
+        <v/>
+      </c>
+      <c r="I103" t="str">
+        <v/>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>komkommertje</v>
+        <v>vanillearoma</v>
       </c>
       <c r="B104" t="str">
-        <v>komkommer</v>
+        <v>vanille extract</v>
+      </c>
+      <c r="C104" t="str">
+        <v>vanilleextract</v>
+      </c>
+      <c r="D104" t="str">
+        <v/>
+      </c>
+      <c r="E104" t="str">
+        <v/>
+      </c>
+      <c r="F104" t="str">
+        <v/>
+      </c>
+      <c r="G104" t="str">
+        <v/>
+      </c>
+      <c r="H104" t="str">
+        <v/>
+      </c>
+      <c r="I104" t="str">
+        <v/>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>verse koriander</v>
+        <v>vanillestokjes</v>
       </c>
       <c r="B105" t="str">
-        <v>koriander</v>
+        <v>vanillestokje</v>
+      </c>
+      <c r="C105" t="str">
+        <v/>
+      </c>
+      <c r="D105" t="str">
+        <v/>
+      </c>
+      <c r="E105" t="str">
+        <v/>
+      </c>
+      <c r="F105" t="str">
+        <v/>
+      </c>
+      <c r="G105" t="str">
+        <v/>
+      </c>
+      <c r="H105" t="str">
+        <v/>
+      </c>
+      <c r="I105" t="str">
+        <v/>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>pasta</v>
+        <v>verse_gist</v>
       </c>
       <c r="B106" t="str">
-        <v>lasagnevellen</v>
+        <v>gist</v>
+      </c>
+      <c r="C106" t="str">
+        <v/>
+      </c>
+      <c r="D106" t="str">
+        <v/>
+      </c>
+      <c r="E106" t="str">
+        <v/>
+      </c>
+      <c r="F106" t="str">
+        <v/>
+      </c>
+      <c r="G106" t="str">
+        <v/>
+      </c>
+      <c r="H106" t="str">
+        <v/>
+      </c>
+      <c r="I106" t="str">
+        <v/>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>laurierblaadjes</v>
+        <v>visbouillon</v>
       </c>
       <c r="B107" t="str">
-        <v>laurier</v>
+        <v>visbouillon</v>
+      </c>
+      <c r="C107" t="str">
+        <v/>
+      </c>
+      <c r="D107" t="str">
+        <v/>
+      </c>
+      <c r="E107" t="str">
+        <v/>
+      </c>
+      <c r="F107" t="str">
+        <v/>
+      </c>
+      <c r="G107" t="str">
+        <v/>
+      </c>
+      <c r="H107" t="str">
+        <v/>
+      </c>
+      <c r="I107" t="str">
+        <v/>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>laurierblad</v>
+        <v>vleesbouillon</v>
       </c>
       <c r="B108" t="str">
-        <v>laurier</v>
+        <v>vleesbouillon</v>
+      </c>
+      <c r="C108" t="str">
+        <v/>
+      </c>
+      <c r="D108" t="str">
+        <v/>
+      </c>
+      <c r="E108" t="str">
+        <v/>
+      </c>
+      <c r="F108" t="str">
+        <v/>
+      </c>
+      <c r="G108" t="str">
+        <v/>
+      </c>
+      <c r="H108" t="str">
+        <v/>
+      </c>
+      <c r="I108" t="str">
+        <v/>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>limoen</v>
+        <v>walnoten</v>
       </c>
       <c r="B109" t="str">
-        <v>limoen</v>
+        <v>walnoot</v>
+      </c>
+      <c r="C109" t="str">
+        <v/>
+      </c>
+      <c r="D109" t="str">
+        <v/>
+      </c>
+      <c r="E109" t="str">
+        <v/>
+      </c>
+      <c r="F109" t="str">
+        <v/>
+      </c>
+      <c r="G109" t="str">
+        <v/>
+      </c>
+      <c r="H109" t="str">
+        <v/>
+      </c>
+      <c r="I109" t="str">
+        <v/>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>limoensap</v>
+        <v>witloof</v>
       </c>
       <c r="B110" t="str">
-        <v>limoen</v>
+        <v>witlof</v>
+      </c>
+      <c r="C110" t="str">
+        <v>witloof</v>
+      </c>
+      <c r="D110" t="str">
+        <v/>
+      </c>
+      <c r="E110" t="str">
+        <v/>
+      </c>
+      <c r="F110" t="str">
+        <v/>
+      </c>
+      <c r="G110" t="str">
+        <v/>
+      </c>
+      <c r="H110" t="str">
+        <v/>
+      </c>
+      <c r="I110" t="str">
+        <v/>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>knoflook</v>
+        <v>witte_wijn</v>
       </c>
       <c r="B111" t="str">
-        <v>look</v>
+        <v>witte wijn</v>
+      </c>
+      <c r="C111" t="str">
+        <v/>
+      </c>
+      <c r="D111" t="str">
+        <v/>
+      </c>
+      <c r="E111" t="str">
+        <v/>
+      </c>
+      <c r="F111" t="str">
+        <v/>
+      </c>
+      <c r="G111" t="str">
+        <v/>
+      </c>
+      <c r="H111" t="str">
+        <v/>
+      </c>
+      <c r="I111" t="str">
+        <v/>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>knoflookteentje</v>
+        <v>wortelen</v>
       </c>
       <c r="B112" t="str">
-        <v>look</v>
+        <v>peen</v>
+      </c>
+      <c r="C112" t="str">
+        <v>penen</v>
+      </c>
+      <c r="D112" t="str">
+        <v>wortel</v>
+      </c>
+      <c r="E112" t="str">
+        <v>wortels</v>
+      </c>
+      <c r="F112" t="str">
+        <v>worteltje</v>
+      </c>
+      <c r="G112" t="str">
+        <v>worteltjes</v>
+      </c>
+      <c r="H112" t="str">
+        <v/>
+      </c>
+      <c r="I112" t="str">
+        <v/>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>knoflookteentjes</v>
+        <v>wraps</v>
       </c>
       <c r="B113" t="str">
-        <v>look</v>
+        <v>tortilla</v>
+      </c>
+      <c r="C113" t="str">
+        <v>wraps</v>
+      </c>
+      <c r="D113" t="str">
+        <v/>
+      </c>
+      <c r="E113" t="str">
+        <v/>
+      </c>
+      <c r="F113" t="str">
+        <v/>
+      </c>
+      <c r="G113" t="str">
+        <v/>
+      </c>
+      <c r="H113" t="str">
+        <v/>
+      </c>
+      <c r="I113" t="str">
+        <v/>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>lookteentje</v>
+        <v>yoghurt</v>
       </c>
       <c r="B114" t="str">
-        <v>look</v>
+        <v>Griekse yoghurt</v>
+      </c>
+      <c r="C114" t="str">
+        <v>yoghurt</v>
+      </c>
+      <c r="D114" t="str">
+        <v/>
+      </c>
+      <c r="E114" t="str">
+        <v/>
+      </c>
+      <c r="F114" t="str">
+        <v/>
+      </c>
+      <c r="G114" t="str">
+        <v/>
+      </c>
+      <c r="H114" t="str">
+        <v/>
+      </c>
+      <c r="I114" t="str">
+        <v/>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>lookteentjes</v>
+        <v>zalm</v>
       </c>
       <c r="B115" t="str">
-        <v>look</v>
+        <v>zalm filet</v>
+      </c>
+      <c r="C115" t="str">
+        <v/>
+      </c>
+      <c r="D115" t="str">
+        <v/>
+      </c>
+      <c r="E115" t="str">
+        <v/>
+      </c>
+      <c r="F115" t="str">
+        <v/>
+      </c>
+      <c r="G115" t="str">
+        <v/>
+      </c>
+      <c r="H115" t="str">
+        <v/>
+      </c>
+      <c r="I115" t="str">
+        <v/>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>teentje knoflook</v>
+        <v>zelfrijzend_bakmeel</v>
       </c>
       <c r="B116" t="str">
-        <v>look</v>
+        <v>bloem</v>
+      </c>
+      <c r="C116" t="str">
+        <v>patentbloem</v>
+      </c>
+      <c r="D116" t="str">
+        <v>tarwebloem</v>
+      </c>
+      <c r="E116" t="str">
+        <v/>
+      </c>
+      <c r="F116" t="str">
+        <v/>
+      </c>
+      <c r="G116" t="str">
+        <v/>
+      </c>
+      <c r="H116" t="str">
+        <v/>
+      </c>
+      <c r="I116" t="str">
+        <v/>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>teentjes knoflook</v>
+        <v>zilveruitjes</v>
       </c>
       <c r="B117" t="str">
-        <v>look</v>
+        <v>kappertje</v>
+      </c>
+      <c r="C117" t="str">
+        <v>zilverui</v>
+      </c>
+      <c r="D117" t="str">
+        <v/>
+      </c>
+      <c r="E117" t="str">
+        <v/>
+      </c>
+      <c r="F117" t="str">
+        <v/>
+      </c>
+      <c r="G117" t="str">
+        <v/>
+      </c>
+      <c r="H117" t="str">
+        <v/>
+      </c>
+      <c r="I117" t="str">
+        <v/>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>mais</v>
+        <v>zoete_aardappelen</v>
       </c>
       <c r="B118" t="str">
-        <v>mais</v>
+        <v>bataat</v>
+      </c>
+      <c r="C118" t="str">
+        <v>zoete aardappel</v>
+      </c>
+      <c r="D118" t="str">
+        <v>zoete aardappels</v>
+      </c>
+      <c r="E118" t="str">
+        <v/>
+      </c>
+      <c r="F118" t="str">
+        <v/>
+      </c>
+      <c r="G118" t="str">
+        <v/>
+      </c>
+      <c r="H118" t="str">
+        <v/>
+      </c>
+      <c r="I118" t="str">
+        <v/>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>maïs</v>
+        <v>zonnebloemolie</v>
       </c>
       <c r="B119" t="str">
-        <v>mais</v>
+        <v>plantaardige olie</v>
+      </c>
+      <c r="C119" t="str">
+        <v>zonnebloem olie</v>
+      </c>
+      <c r="D119" t="str">
+        <v/>
+      </c>
+      <c r="E119" t="str">
+        <v/>
+      </c>
+      <c r="F119" t="str">
+        <v/>
+      </c>
+      <c r="G119" t="str">
+        <v/>
+      </c>
+      <c r="H119" t="str">
+        <v/>
+      </c>
+      <c r="I119" t="str">
+        <v/>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>maiskorrels</v>
+        <v>zure_room</v>
       </c>
       <c r="B120" t="str">
-        <v>mais</v>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="str">
-        <v>maïskorrels</v>
-      </c>
-      <c r="B121" t="str">
-        <v>mais</v>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="str">
-        <v>maïzena</v>
-      </c>
-      <c r="B122" t="str">
-        <v>maizena</v>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="str">
-        <v>zetmeel</v>
-      </c>
-      <c r="B123" t="str">
-        <v>maizena</v>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="str">
-        <v>mandarijn</v>
-      </c>
-      <c r="B124" t="str">
-        <v>mandarijnen</v>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="str">
-        <v>mayonnaise</v>
-      </c>
-      <c r="B125" t="str">
-        <v>mayonaise</v>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="str">
-        <v>halfvolle melk</v>
-      </c>
-      <c r="B126" t="str">
-        <v>melk</v>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="str">
-        <v>volle melk</v>
-      </c>
-      <c r="B127" t="str">
-        <v>melk</v>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="str">
-        <v>mini komkommer</v>
-      </c>
-      <c r="B128" t="str">
-        <v>mini_komkommers</v>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="str">
-        <v>mini komkommers</v>
-      </c>
-      <c r="B129" t="str">
-        <v>mini_komkommers</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="str">
-        <v>dijonmmosterd</v>
-      </c>
-      <c r="B130" t="str">
-        <v>mosterd</v>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="str">
-        <v>mosterd</v>
-      </c>
-      <c r="B131" t="str">
-        <v>mosterd</v>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="str">
-        <v>mozzarella</v>
-      </c>
-      <c r="B132" t="str">
-        <v>mozarella</v>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="str">
-        <v>mozzarelle</v>
-      </c>
-      <c r="B133" t="str">
-        <v>mozarella</v>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="str">
-        <v>verse munt</v>
-      </c>
-      <c r="B134" t="str">
-        <v>munt</v>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="str">
-        <v>extra vergine olijfolie</v>
-      </c>
-      <c r="B135" t="str">
-        <v>olijfolie</v>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="str">
-        <v>olijfolie extra vierge</v>
-      </c>
-      <c r="B136" t="str">
-        <v>olijfolie</v>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="str">
-        <v>paksoy</v>
-      </c>
-      <c r="B137" t="str">
-        <v>paksoi</v>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="str">
-        <v>broodkruim</v>
-      </c>
-      <c r="B138" t="str">
-        <v>paneermeel</v>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="str">
-        <v>broodkruimels</v>
-      </c>
-      <c r="B139" t="str">
-        <v>paneermeel</v>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="str">
-        <v>groene paprika</v>
-      </c>
-      <c r="B140" t="str">
-        <v>paprika</v>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="str">
-        <v>paprika</v>
-      </c>
-      <c r="B141" t="str">
-        <v>paprika</v>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="str">
-        <v>rode paprika</v>
-      </c>
-      <c r="B142" t="str">
-        <v>paprika</v>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="str">
-        <v>parma ham</v>
-      </c>
-      <c r="B143" t="str">
-        <v>parmaham</v>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="str">
-        <v>rauwe ham</v>
-      </c>
-      <c r="B144" t="str">
-        <v>parmaham</v>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="str">
-        <v>parmezaan kaas</v>
-      </c>
-      <c r="B145" t="str">
-        <v>parmezaan</v>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="str">
-        <v>parmezaankaas</v>
-      </c>
-      <c r="B146" t="str">
-        <v>parmezaan</v>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="str">
-        <v>parmezaanse kaas</v>
-      </c>
-      <c r="B147" t="str">
-        <v>parmezaan</v>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="str">
-        <v>passata</v>
-      </c>
-      <c r="B148" t="str">
-        <v>passata</v>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="str">
-        <v>peer</v>
-      </c>
-      <c r="B149" t="str">
-        <v>peren</v>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="str">
-        <v>verse peterselie</v>
-      </c>
-      <c r="B150" t="str">
-        <v>peterselie</v>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="str">
-        <v>bosui</v>
-      </c>
-      <c r="B151" t="str">
-        <v>pijpajuin</v>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="str">
-        <v>bosuitje</v>
-      </c>
-      <c r="B152" t="str">
-        <v>pijpajuin</v>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="str">
-        <v>bosuitjes</v>
-      </c>
-      <c r="B153" t="str">
-        <v>pijpajuin</v>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="str">
-        <v>lente-ui</v>
-      </c>
-      <c r="B154" t="str">
-        <v>pijpajuin</v>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="str">
-        <v>lenteui</v>
-      </c>
-      <c r="B155" t="str">
-        <v>pijpajuin</v>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="str">
-        <v>lenteuitje</v>
-      </c>
-      <c r="B156" t="str">
-        <v>pijpajuin</v>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="str">
-        <v>pijpajuintje</v>
-      </c>
-      <c r="B157" t="str">
-        <v>pijpajuin</v>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="str">
-        <v>kwark</v>
-      </c>
-      <c r="B158" t="str">
-        <v>platte_kaas</v>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="str">
-        <v>platte kaas</v>
-      </c>
-      <c r="B159" t="str">
-        <v>platte_kaas</v>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="str">
-        <v>pudding</v>
-      </c>
-      <c r="B160" t="str">
-        <v>pudding_poeder</v>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="str">
-        <v>puddingpoeder</v>
-      </c>
-      <c r="B161" t="str">
-        <v>pudding_poeder</v>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="str">
-        <v>radijs</v>
-      </c>
-      <c r="B162" t="str">
-        <v>radijsjes</v>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" t="str">
-        <v>radiJs</v>
-      </c>
-      <c r="B163" t="str">
-        <v>radijsjes</v>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" t="str">
-        <v>rijstvellen</v>
-      </c>
-      <c r="B164" t="str">
-        <v>rijstpapier</v>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" t="str">
-        <v>rode ajuin</v>
-      </c>
-      <c r="B165" t="str">
-        <v>rode_ajuin</v>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" t="str">
-        <v>rode ui</v>
-      </c>
-      <c r="B166" t="str">
-        <v>rode_ajuin</v>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" t="str">
-        <v>rode uien</v>
-      </c>
-      <c r="B167" t="str">
-        <v>rode_ajuin</v>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" t="str">
-        <v>currypasta</v>
-      </c>
-      <c r="B168" t="str">
-        <v>rode_currypasta</v>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" t="str">
-        <v>rode wijn</v>
-      </c>
-      <c r="B169" t="str">
-        <v>rode_wijn</v>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" t="str">
-        <v>room</v>
-      </c>
-      <c r="B170" t="str">
-        <v>room</v>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" t="str">
-        <v>slagroom</v>
-      </c>
-      <c r="B171" t="str">
-        <v>room</v>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" t="str">
-        <v>verse rozemarijn</v>
-      </c>
-      <c r="B172" t="str">
-        <v>rozemarijn</v>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="str">
-        <v>runderbouillon</v>
-      </c>
-      <c r="B173" t="str">
-        <v>rundsbouillon</v>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="str">
-        <v>satékruiden</v>
-      </c>
-      <c r="B174" t="str">
-        <v>satekruiden</v>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="str">
-        <v>satésaus</v>
-      </c>
-      <c r="B175" t="str">
-        <v>satekruiden</v>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="str">
-        <v>oester</v>
-      </c>
-      <c r="B176" t="str">
-        <v>scampis</v>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="str">
-        <v>scampi</v>
-      </c>
-      <c r="B177" t="str">
-        <v>scampis</v>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="str">
-        <v>selderie</v>
-      </c>
-      <c r="B178" t="str">
-        <v>selder</v>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="str">
-        <v>selderij</v>
-      </c>
-      <c r="B179" t="str">
-        <v>selder</v>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="str">
-        <v>sesamolie</v>
-      </c>
-      <c r="B180" t="str">
-        <v>sesamolie</v>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="str">
-        <v>sjalot</v>
-      </c>
-      <c r="B181" t="str">
-        <v>sjalotten</v>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="str">
-        <v>sjalotje</v>
-      </c>
-      <c r="B182" t="str">
-        <v>sjalotten</v>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="str">
-        <v>sjalotjes</v>
-      </c>
-      <c r="B183" t="str">
-        <v>sjalotten</v>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="str">
-        <v>soja saus</v>
-      </c>
-      <c r="B184" t="str">
-        <v>sojasaus</v>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="str">
-        <v>sojasaus</v>
-      </c>
-      <c r="B185" t="str">
-        <v>sojasaus</v>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="str">
-        <v>lardons</v>
-      </c>
-      <c r="B186" t="str">
-        <v>spekblokjes</v>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" t="str">
-        <v>spekblokje</v>
-      </c>
-      <c r="B187" t="str">
-        <v>spekblokjes</v>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" t="str">
-        <v>speltmeel</v>
-      </c>
-      <c r="B188" t="str">
-        <v>speltbloem</v>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" t="str">
-        <v>fijne suiker</v>
-      </c>
-      <c r="B189" t="str">
-        <v>suiker</v>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" t="str">
-        <v>kristalsuiker</v>
-      </c>
-      <c r="B190" t="str">
-        <v>suiker</v>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" t="str">
-        <v>suikerklontje</v>
-      </c>
-      <c r="B191" t="str">
-        <v>suikerklontjes</v>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" t="str">
-        <v>verse tijm</v>
-      </c>
-      <c r="B192" t="str">
-        <v>tijm</v>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" t="str">
-        <v>tomaat</v>
-      </c>
-      <c r="B193" t="str">
-        <v>tomaten</v>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="str">
-        <v>tomaatje</v>
-      </c>
-      <c r="B194" t="str">
-        <v>tomaten</v>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="str">
-        <v>tomaten uit blik</v>
-      </c>
-      <c r="B195" t="str">
-        <v>tomaten_uit_blik</v>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" t="str">
-        <v>tomatenblokjes</v>
-      </c>
-      <c r="B196" t="str">
-        <v>tomatenblokjes</v>
-      </c>
-    </row>
-    <row r="197">
-      <c r="A197" t="str">
-        <v>geconcentreerde tomatenpuree</v>
-      </c>
-      <c r="B197" t="str">
-        <v>tomatenpuree</v>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" t="str">
-        <v>tomatenpuree</v>
-      </c>
-      <c r="B198" t="str">
-        <v>tomatenpuree</v>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" t="str">
-        <v>vanille extract</v>
-      </c>
-      <c r="B199" t="str">
-        <v>vanillearoma</v>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" t="str">
-        <v>vanilleextract</v>
-      </c>
-      <c r="B200" t="str">
-        <v>vanillearoma</v>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" t="str">
-        <v>vanillestokje</v>
-      </c>
-      <c r="B201" t="str">
-        <v>vanillestokjes</v>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" t="str">
-        <v>gist</v>
-      </c>
-      <c r="B202" t="str">
-        <v>verse_gist</v>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" t="str">
-        <v>visbouillon</v>
-      </c>
-      <c r="B203" t="str">
-        <v>visbouillon</v>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" t="str">
-        <v>vleesbouillon</v>
-      </c>
-      <c r="B204" t="str">
-        <v>vleesbouillon</v>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" t="str">
-        <v>walnoot</v>
-      </c>
-      <c r="B205" t="str">
-        <v>walnoten</v>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" t="str">
-        <v>witlof</v>
-      </c>
-      <c r="B206" t="str">
-        <v>witloof</v>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" t="str">
-        <v>witloof</v>
-      </c>
-      <c r="B207" t="str">
-        <v>witloof</v>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" t="str">
-        <v>witte wijn</v>
-      </c>
-      <c r="B208" t="str">
-        <v>witte_wijn</v>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" t="str">
-        <v>peen</v>
-      </c>
-      <c r="B209" t="str">
-        <v>wortelen</v>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" t="str">
-        <v>penen</v>
-      </c>
-      <c r="B210" t="str">
-        <v>wortelen</v>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" t="str">
-        <v>wortel</v>
-      </c>
-      <c r="B211" t="str">
-        <v>wortelen</v>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" t="str">
-        <v>wortels</v>
-      </c>
-      <c r="B212" t="str">
-        <v>wortelen</v>
-      </c>
-    </row>
-    <row r="213">
-      <c r="A213" t="str">
-        <v>worteltje</v>
-      </c>
-      <c r="B213" t="str">
-        <v>wortelen</v>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" t="str">
-        <v>worteltjes</v>
-      </c>
-      <c r="B214" t="str">
-        <v>wortelen</v>
-      </c>
-    </row>
-    <row r="215">
-      <c r="A215" t="str">
-        <v>tortilla</v>
-      </c>
-      <c r="B215" t="str">
-        <v>wraps</v>
-      </c>
-    </row>
-    <row r="216">
-      <c r="A216" t="str">
-        <v>wraps</v>
-      </c>
-      <c r="B216" t="str">
-        <v>wraps</v>
-      </c>
-    </row>
-    <row r="217">
-      <c r="A217" t="str">
-        <v>Griekse yoghurt</v>
-      </c>
-      <c r="B217" t="str">
-        <v>yoghurt</v>
-      </c>
-    </row>
-    <row r="218">
-      <c r="A218" t="str">
-        <v>yoghurt</v>
-      </c>
-      <c r="B218" t="str">
-        <v>yoghurt</v>
-      </c>
-    </row>
-    <row r="219">
-      <c r="A219" t="str">
-        <v>zalm filet</v>
-      </c>
-      <c r="B219" t="str">
-        <v>zalm</v>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" t="str">
-        <v>bloem</v>
-      </c>
-      <c r="B220" t="str">
-        <v>zelfrijzend_bakmeel</v>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" t="str">
-        <v>patentbloem</v>
-      </c>
-      <c r="B221" t="str">
-        <v>zelfrijzend_bakmeel</v>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" t="str">
-        <v>tarwebloem</v>
-      </c>
-      <c r="B222" t="str">
-        <v>zelfrijzend_bakmeel</v>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" t="str">
-        <v>kappertje</v>
-      </c>
-      <c r="B223" t="str">
-        <v>zilveruitjes</v>
-      </c>
-    </row>
-    <row r="224">
-      <c r="A224" t="str">
-        <v>zilverui</v>
-      </c>
-      <c r="B224" t="str">
-        <v>zilveruitjes</v>
-      </c>
-    </row>
-    <row r="225">
-      <c r="A225" t="str">
-        <v>bataat</v>
-      </c>
-      <c r="B225" t="str">
-        <v>zoete_aardappelen</v>
-      </c>
-    </row>
-    <row r="226">
-      <c r="A226" t="str">
-        <v>zoete aardappel</v>
-      </c>
-      <c r="B226" t="str">
-        <v>zoete_aardappelen</v>
-      </c>
-    </row>
-    <row r="227">
-      <c r="A227" t="str">
-        <v>zoete aardappels</v>
-      </c>
-      <c r="B227" t="str">
-        <v>zoete_aardappelen</v>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" t="str">
-        <v>plantaardige olie</v>
-      </c>
-      <c r="B228" t="str">
-        <v>zonnebloemolie</v>
-      </c>
-    </row>
-    <row r="229">
-      <c r="A229" t="str">
-        <v>zonnebloem olie</v>
-      </c>
-      <c r="B229" t="str">
-        <v>zonnebloemolie</v>
-      </c>
-    </row>
-    <row r="230">
-      <c r="A230" t="str">
         <v>zure room</v>
       </c>
-      <c r="B230" t="str">
-        <v>zure_room</v>
+      <c r="C120" t="str">
+        <v/>
+      </c>
+      <c r="D120" t="str">
+        <v/>
+      </c>
+      <c r="E120" t="str">
+        <v/>
+      </c>
+      <c r="F120" t="str">
+        <v/>
+      </c>
+      <c r="G120" t="str">
+        <v/>
+      </c>
+      <c r="H120" t="str">
+        <v/>
+      </c>
+      <c r="I120" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B230"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I120"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: mobiel naam-autocomplete — toetsenbord en focus bij slide-in
- Slide-in: useLayoutEffect, directe focus + transitionend-back-up, autoFocus
- Trigger: flushSync zodat focus binnen user-activation blijft
- Excel workbook meegecommit (lokale wijziging)

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/public/images/items/ingredienten_categorieen.xlsx
+++ b/public/images/items/ingredienten_categorieen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kristoflesaffre/Downloads/ShoppingList/public/images/items/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDFCB3C2-1DAB-4A43-A1BA-33678E0F3BB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59CD2604-FFC0-CA45-B59F-935B7448D7B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="20200" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="896" uniqueCount="514">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="897" uniqueCount="515">
   <si>
     <t>Categorie</t>
   </si>
@@ -1568,6 +1568,9 @@
   </si>
   <si>
     <t>kruiden</t>
+  </si>
+  <si>
+    <t>bou</t>
   </si>
 </sst>
 </file>
@@ -5393,7 +5396,9 @@
       <c r="B48" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="C48" s="38"/>
+      <c r="C48" s="38" t="s">
+        <v>514</v>
+      </c>
       <c r="D48" s="38"/>
       <c r="E48" s="38"/>
       <c r="F48" s="38"/>

</xml_diff>